<commit_message>
🔒 [FULL] Daily chip data 2026-05-23 14:13
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-05-22.xlsx
+++ b/data/reports/chip_radar_2026-05-22.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L462"/>
+  <dimension ref="A1:L472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19.28515625" customWidth="1" min="1" max="1"/>
@@ -15750,110 +15750,65 @@
       </c>
     </row>
     <row r="441" ht="16.5" customHeight="1">
-      <c r="A441" s="1" t="inlineStr">
-        <is>
-          <t>高手</t>
-        </is>
-      </c>
-      <c r="B441" s="1" t="inlineStr">
-        <is>
-          <t>分點</t>
-        </is>
-      </c>
-      <c r="C441" s="1" t="inlineStr">
-        <is>
-          <t>代號</t>
-        </is>
-      </c>
-      <c r="D441" s="1" t="inlineStr">
-        <is>
-          <t>標的</t>
-        </is>
-      </c>
-      <c r="E441" s="1" t="inlineStr">
-        <is>
-          <t>買進(張)</t>
-        </is>
-      </c>
-      <c r="F441" s="1" t="inlineStr">
-        <is>
-          <t>賣出(張)</t>
-        </is>
-      </c>
-      <c r="G441" s="1" t="inlineStr">
-        <is>
-          <t>買進(萬元)</t>
-        </is>
-      </c>
-      <c r="H441" s="1" t="inlineStr">
-        <is>
-          <t>賣出(萬元)</t>
-        </is>
-      </c>
-      <c r="I441" s="1" t="inlineStr">
-        <is>
-          <t>淨買差(萬元)</t>
-        </is>
-      </c>
-      <c r="J441" s="1" t="inlineStr">
-        <is>
-          <t>買均</t>
-        </is>
-      </c>
-      <c r="K441" s="1" t="inlineStr">
-        <is>
-          <t>賣均</t>
-        </is>
-      </c>
-      <c r="L441" s="1" t="inlineStr">
-        <is>
-          <t>損益(萬)</t>
-        </is>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>頎邦(6147)</t>
+        </is>
+      </c>
+      <c r="E441" s="3" t="n">
+        <v>121</v>
+      </c>
+      <c r="F441" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="G441" s="3" t="n">
+        <v>2670</v>
+      </c>
+      <c r="H441" s="3" t="n">
+        <v>1592</v>
+      </c>
+      <c r="I441" s="3" t="n">
+        <v>1078</v>
+      </c>
+      <c r="J441" s="4" t="n">
+        <v>220.64</v>
+      </c>
+      <c r="K441" s="4" t="n">
+        <v>218.1</v>
+      </c>
+      <c r="L441" s="6">
+        <f>F441*(K441-J441)</f>
+        <v/>
       </c>
     </row>
     <row r="442" ht="16.5" customHeight="1">
-      <c r="A442" s="1" t="inlineStr">
-        <is>
-          <t>竹科主力分點</t>
-        </is>
-      </c>
-      <c r="B442" s="1" t="inlineStr">
-        <is>
-          <t>兆豐-新竹</t>
-        </is>
-      </c>
-      <c r="C442" s="1" t="inlineStr">
-        <is>
-          <t>700V</t>
-        </is>
-      </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>睿生光電(6861)</t>
+          <t>騰輝電子-KY(6672)</t>
         </is>
       </c>
       <c r="E442" s="3" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="F442" s="3" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="G442" s="3" t="n">
-        <v>5803</v>
+        <v>2606</v>
       </c>
       <c r="H442" s="3" t="n">
-        <v>2468</v>
+        <v>1550</v>
       </c>
       <c r="I442" s="3" t="n">
-        <v>3335</v>
+        <v>1056</v>
       </c>
       <c r="J442" s="4" t="n">
-        <v>436.33</v>
+        <v>188.88</v>
       </c>
       <c r="K442" s="4" t="n">
-        <v>432.96</v>
-      </c>
-      <c r="L442" s="6">
+        <v>193.71</v>
+      </c>
+      <c r="L442" s="5">
         <f>F442*(K442-J442)</f>
         <v/>
       </c>
@@ -15861,31 +15816,31 @@
     <row r="443" ht="16.5" customHeight="1">
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>合勤控(3704)</t>
+          <t>台灣大(3045)</t>
         </is>
       </c>
       <c r="E443" s="3" t="n">
-        <v>1135</v>
+        <v>190</v>
       </c>
       <c r="F443" s="3" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="G443" s="3" t="n">
-        <v>4824</v>
+        <v>2128</v>
       </c>
       <c r="H443" s="3" t="n">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="I443" s="3" t="n">
-        <v>4480</v>
+        <v>1792</v>
       </c>
       <c r="J443" s="4" t="n">
-        <v>42.51</v>
+        <v>112.03</v>
       </c>
       <c r="K443" s="4" t="n">
-        <v>43.01</v>
-      </c>
-      <c r="L443" s="5">
+        <v>112</v>
+      </c>
+      <c r="L443" s="6">
         <f>F443*(K443-J443)</f>
         <v/>
       </c>
@@ -15893,31 +15848,31 @@
     <row r="444" ht="16.5" customHeight="1">
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>啟��(6285)</t>
+          <t>新唐(4919)</t>
         </is>
       </c>
       <c r="E444" s="3" t="n">
-        <v>163</v>
+        <v>102</v>
       </c>
       <c r="F444" s="3" t="n">
-        <v>111</v>
+        <v>70</v>
       </c>
       <c r="G444" s="3" t="n">
-        <v>4680</v>
+        <v>2040</v>
       </c>
       <c r="H444" s="3" t="n">
-        <v>3259</v>
+        <v>1393</v>
       </c>
       <c r="I444" s="3" t="n">
-        <v>1421</v>
+        <v>647</v>
       </c>
       <c r="J444" s="4" t="n">
-        <v>287.15</v>
+        <v>199.98</v>
       </c>
       <c r="K444" s="4" t="n">
-        <v>293.59</v>
-      </c>
-      <c r="L444" s="5">
+        <v>199.04</v>
+      </c>
+      <c r="L444" s="6">
         <f>F444*(K444-J444)</f>
         <v/>
       </c>
@@ -15925,29 +15880,29 @@
     <row r="445" ht="16.5" customHeight="1">
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>宜鼎(5289)</t>
         </is>
       </c>
       <c r="E445" s="3" t="n">
-        <v>320</v>
+        <v>10</v>
       </c>
       <c r="F445" s="3" t="n">
-        <v>208</v>
+        <v>7</v>
       </c>
       <c r="G445" s="3" t="n">
-        <v>3653</v>
+        <v>1666</v>
       </c>
       <c r="H445" s="3" t="n">
-        <v>2381</v>
+        <v>1167</v>
       </c>
       <c r="I445" s="3" t="n">
-        <v>1272</v>
+        <v>499</v>
       </c>
       <c r="J445" s="4" t="n">
-        <v>114.15</v>
+        <v>1666</v>
       </c>
       <c r="K445" s="4" t="n">
-        <v>114.45</v>
+        <v>1666.71</v>
       </c>
       <c r="L445" s="5">
         <f>F445*(K445-J445)</f>
@@ -15957,29 +15912,29 @@
     <row r="446" ht="16.5" customHeight="1">
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>欣興(3037)</t>
+          <t>期元大道瓊白銀(00738U)</t>
         </is>
       </c>
       <c r="E446" s="3" t="n">
-        <v>34</v>
+        <v>240</v>
       </c>
       <c r="F446" s="3" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="G446" s="3" t="n">
-        <v>3296</v>
+        <v>1476</v>
       </c>
       <c r="H446" s="3" t="n">
-        <v>2138</v>
+        <v>31</v>
       </c>
       <c r="I446" s="3" t="n">
-        <v>1158</v>
+        <v>1445</v>
       </c>
       <c r="J446" s="4" t="n">
-        <v>969.53</v>
+        <v>61.49</v>
       </c>
       <c r="K446" s="4" t="n">
-        <v>971.73</v>
+        <v>62.4</v>
       </c>
       <c r="L446" s="5">
         <f>F446*(K446-J446)</f>
@@ -15989,29 +15944,29 @@
     <row r="447" ht="16.5" customHeight="1">
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>群聯(8299)</t>
+          <t>智原(3035)</t>
         </is>
       </c>
       <c r="E447" s="3" t="n">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="F447" s="3" t="n">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="G447" s="3" t="n">
-        <v>2833</v>
+        <v>1432</v>
       </c>
       <c r="H447" s="3" t="n">
-        <v>1839</v>
+        <v>881</v>
       </c>
       <c r="I447" s="3" t="n">
-        <v>994</v>
+        <v>551</v>
       </c>
       <c r="J447" s="4" t="n">
-        <v>2360.58</v>
+        <v>210.59</v>
       </c>
       <c r="K447" s="4" t="n">
-        <v>2298.88</v>
+        <v>209.79</v>
       </c>
       <c r="L447" s="6">
         <f>F447*(K447-J447)</f>
@@ -16021,31 +15976,31 @@
     <row r="448" ht="16.5" customHeight="1">
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>奇鋐(3017)</t>
+          <t>晶技(3042)</t>
         </is>
       </c>
       <c r="E448" s="3" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="F448" s="3" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="G448" s="3" t="n">
-        <v>2137</v>
+        <v>1415</v>
       </c>
       <c r="H448" s="3" t="n">
-        <v>1589</v>
+        <v>885</v>
       </c>
       <c r="I448" s="3" t="n">
-        <v>548</v>
+        <v>530</v>
       </c>
       <c r="J448" s="4" t="n">
-        <v>2670.75</v>
+        <v>176.91</v>
       </c>
       <c r="K448" s="4" t="n">
-        <v>2648.33</v>
-      </c>
-      <c r="L448" s="6">
+        <v>176.92</v>
+      </c>
+      <c r="L448" s="5">
         <f>F448*(K448-J448)</f>
         <v/>
       </c>
@@ -16053,29 +16008,29 @@
     <row r="449" ht="16.5" customHeight="1">
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>聯鈞(3450)</t>
+          <t>敬鵬(2355)</t>
         </is>
       </c>
       <c r="E449" s="3" t="n">
-        <v>30</v>
+        <v>204</v>
       </c>
       <c r="F449" s="3" t="n">
-        <v>2</v>
+        <v>133</v>
       </c>
       <c r="G449" s="3" t="n">
-        <v>1364</v>
+        <v>1330</v>
       </c>
       <c r="H449" s="3" t="n">
-        <v>92</v>
+        <v>867</v>
       </c>
       <c r="I449" s="3" t="n">
-        <v>1272</v>
+        <v>463</v>
       </c>
       <c r="J449" s="4" t="n">
-        <v>454.6</v>
+        <v>65.2</v>
       </c>
       <c r="K449" s="4" t="n">
-        <v>462</v>
+        <v>65.2</v>
       </c>
       <c r="L449" s="5">
         <f>F449*(K449-J449)</f>
@@ -16085,162 +16040,172 @@
     <row r="450" ht="16.5" customHeight="1">
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>京元電子(2449)</t>
+          <t>中租-KY(5871)</t>
         </is>
       </c>
       <c r="E450" s="3" t="n">
-        <v>36</v>
+        <v>116</v>
       </c>
       <c r="F450" s="3" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="G450" s="3" t="n">
-        <v>1051</v>
+        <v>1291</v>
       </c>
       <c r="H450" s="3" t="n">
-        <v>407</v>
+        <v>359</v>
       </c>
       <c r="I450" s="3" t="n">
-        <v>644</v>
+        <v>932</v>
       </c>
       <c r="J450" s="4" t="n">
-        <v>292.06</v>
+        <v>111.3</v>
       </c>
       <c r="K450" s="4" t="n">
-        <v>290.86</v>
-      </c>
-      <c r="L450" s="6">
+        <v>112.31</v>
+      </c>
+      <c r="L450" s="5">
         <f>F450*(K450-J450)</f>
         <v/>
       </c>
     </row>
     <row r="451" ht="16.5" customHeight="1">
-      <c r="D451" s="2" t="inlineStr">
-        <is>
-          <t>聯詠(3034)</t>
-        </is>
-      </c>
-      <c r="E451" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="F451" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G451" s="3" t="n">
-        <v>1026</v>
-      </c>
-      <c r="H451" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="I451" s="3" t="n">
-        <v>1009</v>
-      </c>
-      <c r="J451" s="4" t="n">
-        <v>488.67</v>
-      </c>
-      <c r="K451" s="4" t="n">
-        <v>174</v>
-      </c>
-      <c r="L451" s="6">
-        <f>F451*(K451-J451)</f>
-        <v/>
+      <c r="A451" s="1" t="inlineStr">
+        <is>
+          <t>高手</t>
+        </is>
+      </c>
+      <c r="B451" s="1" t="inlineStr">
+        <is>
+          <t>分點</t>
+        </is>
+      </c>
+      <c r="C451" s="1" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="D451" s="1" t="inlineStr">
+        <is>
+          <t>標的</t>
+        </is>
+      </c>
+      <c r="E451" s="1" t="inlineStr">
+        <is>
+          <t>買進(張)</t>
+        </is>
+      </c>
+      <c r="F451" s="1" t="inlineStr">
+        <is>
+          <t>賣出(張)</t>
+        </is>
+      </c>
+      <c r="G451" s="1" t="inlineStr">
+        <is>
+          <t>買進(萬元)</t>
+        </is>
+      </c>
+      <c r="H451" s="1" t="inlineStr">
+        <is>
+          <t>賣出(萬元)</t>
+        </is>
+      </c>
+      <c r="I451" s="1" t="inlineStr">
+        <is>
+          <t>淨買差(萬元)</t>
+        </is>
+      </c>
+      <c r="J451" s="1" t="inlineStr">
+        <is>
+          <t>買均</t>
+        </is>
+      </c>
+      <c r="K451" s="1" t="inlineStr">
+        <is>
+          <t>賣均</t>
+        </is>
+      </c>
+      <c r="L451" s="1" t="inlineStr">
+        <is>
+          <t>損益(萬)</t>
+        </is>
       </c>
     </row>
     <row r="452" ht="16.5" customHeight="1">
+      <c r="A452" s="1" t="inlineStr">
+        <is>
+          <t>竹科主力分點</t>
+        </is>
+      </c>
       <c r="B452" s="1" t="inlineStr">
         <is>
-          <t>分點</t>
+          <t>兆豐-新竹</t>
         </is>
       </c>
       <c r="C452" s="1" t="inlineStr">
         <is>
-          <t>代號</t>
-        </is>
-      </c>
-      <c r="D452" s="1" t="inlineStr">
-        <is>
-          <t>標的</t>
-        </is>
-      </c>
-      <c r="E452" s="1" t="inlineStr">
-        <is>
-          <t>買進(張)</t>
-        </is>
-      </c>
-      <c r="F452" s="1" t="inlineStr">
-        <is>
-          <t>賣出(張)</t>
-        </is>
-      </c>
-      <c r="G452" s="1" t="inlineStr">
-        <is>
-          <t>買進(萬元)</t>
-        </is>
-      </c>
-      <c r="H452" s="1" t="inlineStr">
-        <is>
-          <t>賣出(萬元)</t>
-        </is>
-      </c>
-      <c r="I452" s="1" t="inlineStr">
-        <is>
-          <t>淨買差(萬元)</t>
-        </is>
-      </c>
-      <c r="J452" s="1" t="inlineStr">
-        <is>
-          <t>買均</t>
-        </is>
-      </c>
-      <c r="K452" s="1" t="inlineStr">
-        <is>
-          <t>賣均</t>
-        </is>
-      </c>
-      <c r="L452" s="1" t="inlineStr">
-        <is>
-          <t>損益(萬)</t>
-        </is>
+          <t>700V</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>睿生光電(6861)</t>
+        </is>
+      </c>
+      <c r="E452" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="F452" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="G452" s="3" t="n">
+        <v>5803</v>
+      </c>
+      <c r="H452" s="3" t="n">
+        <v>2468</v>
+      </c>
+      <c r="I452" s="3" t="n">
+        <v>3335</v>
+      </c>
+      <c r="J452" s="4" t="n">
+        <v>436.33</v>
+      </c>
+      <c r="K452" s="4" t="n">
+        <v>432.96</v>
+      </c>
+      <c r="L452" s="6">
+        <f>F452*(K452-J452)</f>
+        <v/>
       </c>
     </row>
     <row r="453" ht="16.5" customHeight="1">
-      <c r="B453" s="1" t="inlineStr">
-        <is>
-          <t>富邦-新竹</t>
-        </is>
-      </c>
-      <c r="C453" s="1" t="inlineStr">
-        <is>
-          <t>9647</t>
-        </is>
-      </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>合勤控(3704)</t>
         </is>
       </c>
       <c r="E453" s="3" t="n">
-        <v>35</v>
+        <v>1135</v>
       </c>
       <c r="F453" s="3" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="G453" s="3" t="n">
-        <v>7959</v>
+        <v>4824</v>
       </c>
       <c r="H453" s="3" t="n">
-        <v>6776</v>
+        <v>344</v>
       </c>
       <c r="I453" s="3" t="n">
-        <v>1183</v>
+        <v>4480</v>
       </c>
       <c r="J453" s="4" t="n">
-        <v>2273.89</v>
+        <v>42.51</v>
       </c>
       <c r="K453" s="4" t="n">
-        <v>2258.57</v>
-      </c>
-      <c r="L453" s="6">
+        <v>43.01</v>
+      </c>
+      <c r="L453" s="5">
         <f>F453*(K453-J453)</f>
         <v/>
       </c>
@@ -16248,31 +16213,31 @@
     <row r="454" ht="16.5" customHeight="1">
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>群聯(8299)</t>
+          <t>啟��(6285)</t>
         </is>
       </c>
       <c r="E454" s="3" t="n">
-        <v>33</v>
+        <v>163</v>
       </c>
       <c r="F454" s="3" t="n">
-        <v>10</v>
+        <v>111</v>
       </c>
       <c r="G454" s="3" t="n">
-        <v>7921</v>
+        <v>4680</v>
       </c>
       <c r="H454" s="3" t="n">
-        <v>2336</v>
+        <v>3259</v>
       </c>
       <c r="I454" s="3" t="n">
-        <v>5585</v>
+        <v>1421</v>
       </c>
       <c r="J454" s="4" t="n">
-        <v>2400.18</v>
+        <v>287.15</v>
       </c>
       <c r="K454" s="4" t="n">
-        <v>2336.3</v>
-      </c>
-      <c r="L454" s="6">
+        <v>293.59</v>
+      </c>
+      <c r="L454" s="5">
         <f>F454*(K454-J454)</f>
         <v/>
       </c>
@@ -16280,29 +16245,29 @@
     <row r="455" ht="16.5" customHeight="1">
       <c r="D455" s="2" t="inlineStr">
         <is>
-          <t>華通(2313)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E455" s="3" t="n">
-        <v>193</v>
+        <v>320</v>
       </c>
       <c r="F455" s="3" t="n">
-        <v>166</v>
+        <v>208</v>
       </c>
       <c r="G455" s="3" t="n">
-        <v>5352</v>
+        <v>3653</v>
       </c>
       <c r="H455" s="3" t="n">
-        <v>4610</v>
+        <v>2381</v>
       </c>
       <c r="I455" s="3" t="n">
-        <v>742</v>
+        <v>1272</v>
       </c>
       <c r="J455" s="4" t="n">
-        <v>277.3</v>
+        <v>114.15</v>
       </c>
       <c r="K455" s="4" t="n">
-        <v>277.73</v>
+        <v>114.45</v>
       </c>
       <c r="L455" s="5">
         <f>F455*(K455-J455)</f>
@@ -16312,31 +16277,31 @@
     <row r="456" ht="16.5" customHeight="1">
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>欣興(3037)</t>
         </is>
       </c>
       <c r="E456" s="3" t="n">
-        <v>361</v>
+        <v>34</v>
       </c>
       <c r="F456" s="3" t="n">
-        <v>263</v>
+        <v>22</v>
       </c>
       <c r="G456" s="3" t="n">
-        <v>4151</v>
+        <v>3296</v>
       </c>
       <c r="H456" s="3" t="n">
-        <v>3020</v>
+        <v>2138</v>
       </c>
       <c r="I456" s="3" t="n">
-        <v>1131</v>
+        <v>1158</v>
       </c>
       <c r="J456" s="4" t="n">
-        <v>114.99</v>
+        <v>969.53</v>
       </c>
       <c r="K456" s="4" t="n">
-        <v>114.81</v>
-      </c>
-      <c r="L456" s="6">
+        <v>971.73</v>
+      </c>
+      <c r="L456" s="5">
         <f>F456*(K456-J456)</f>
         <v/>
       </c>
@@ -16344,31 +16309,31 @@
     <row r="457" ht="16.5" customHeight="1">
       <c r="D457" s="2" t="inlineStr">
         <is>
-          <t>新代(7750)</t>
+          <t>群聯(8299)</t>
         </is>
       </c>
       <c r="E457" s="3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F457" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G457" s="3" t="n">
-        <v>4138</v>
+        <v>2833</v>
       </c>
       <c r="H457" s="3" t="n">
-        <v>590</v>
+        <v>1839</v>
       </c>
       <c r="I457" s="3" t="n">
-        <v>3548</v>
+        <v>994</v>
       </c>
       <c r="J457" s="4" t="n">
-        <v>2433.88</v>
+        <v>2360.58</v>
       </c>
       <c r="K457" s="4" t="n">
-        <v>2951.5</v>
-      </c>
-      <c r="L457" s="5">
+        <v>2298.88</v>
+      </c>
+      <c r="L457" s="6">
         <f>F457*(K457-J457)</f>
         <v/>
       </c>
@@ -16376,29 +16341,29 @@
     <row r="458" ht="16.5" customHeight="1">
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>主動統一台股增長(00981A)</t>
+          <t>奇鋐(3017)</t>
         </is>
       </c>
       <c r="E458" s="3" t="n">
-        <v>1208</v>
+        <v>8</v>
       </c>
       <c r="F458" s="3" t="n">
-        <v>768</v>
+        <v>6</v>
       </c>
       <c r="G458" s="3" t="n">
-        <v>3601</v>
+        <v>2137</v>
       </c>
       <c r="H458" s="3" t="n">
-        <v>2283</v>
+        <v>1589</v>
       </c>
       <c r="I458" s="3" t="n">
-        <v>1318</v>
+        <v>548</v>
       </c>
       <c r="J458" s="4" t="n">
-        <v>29.81</v>
+        <v>2670.75</v>
       </c>
       <c r="K458" s="4" t="n">
-        <v>29.73</v>
+        <v>2648.33</v>
       </c>
       <c r="L458" s="6">
         <f>F458*(K458-J458)</f>
@@ -16408,31 +16373,31 @@
     <row r="459" ht="16.5" customHeight="1">
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>晶呈科技(4768)</t>
+          <t>聯鈞(3450)</t>
         </is>
       </c>
       <c r="E459" s="3" t="n">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="F459" s="3" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="G459" s="3" t="n">
-        <v>3053</v>
+        <v>1364</v>
       </c>
       <c r="H459" s="3" t="n">
-        <v>1729</v>
+        <v>92</v>
       </c>
       <c r="I459" s="3" t="n">
-        <v>1324</v>
+        <v>1272</v>
       </c>
       <c r="J459" s="4" t="n">
-        <v>455.66</v>
+        <v>454.6</v>
       </c>
       <c r="K459" s="4" t="n">
-        <v>455</v>
-      </c>
-      <c r="L459" s="6">
+        <v>462</v>
+      </c>
+      <c r="L459" s="5">
         <f>F459*(K459-J459)</f>
         <v/>
       </c>
@@ -16440,31 +16405,31 @@
     <row r="460" ht="16.5" customHeight="1">
       <c r="D460" s="2" t="inlineStr">
         <is>
-          <t>睿生光電(6861)</t>
+          <t>京元電子(2449)</t>
         </is>
       </c>
       <c r="E460" s="3" t="n">
-        <v>66</v>
+        <v>36</v>
       </c>
       <c r="F460" s="3" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="G460" s="3" t="n">
-        <v>2961</v>
+        <v>1051</v>
       </c>
       <c r="H460" s="3" t="n">
-        <v>2086</v>
+        <v>407</v>
       </c>
       <c r="I460" s="3" t="n">
-        <v>875</v>
+        <v>644</v>
       </c>
       <c r="J460" s="4" t="n">
-        <v>448.58</v>
+        <v>292.06</v>
       </c>
       <c r="K460" s="4" t="n">
-        <v>453.54</v>
-      </c>
-      <c r="L460" s="5">
+        <v>290.86</v>
+      </c>
+      <c r="L460" s="6">
         <f>F460*(K460-J460)</f>
         <v/>
       </c>
@@ -16472,85 +16437,440 @@
     <row r="461" ht="16.5" customHeight="1">
       <c r="D461" s="2" t="inlineStr">
         <is>
+          <t>聯詠(3034)</t>
+        </is>
+      </c>
+      <c r="E461" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F461" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G461" s="3" t="n">
+        <v>1026</v>
+      </c>
+      <c r="H461" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="I461" s="3" t="n">
+        <v>1009</v>
+      </c>
+      <c r="J461" s="4" t="n">
+        <v>488.67</v>
+      </c>
+      <c r="K461" s="4" t="n">
+        <v>174</v>
+      </c>
+      <c r="L461" s="6">
+        <f>F461*(K461-J461)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="462" ht="16.5" customHeight="1">
+      <c r="B462" s="1" t="inlineStr">
+        <is>
+          <t>分點</t>
+        </is>
+      </c>
+      <c r="C462" s="1" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="D462" s="1" t="inlineStr">
+        <is>
+          <t>標的</t>
+        </is>
+      </c>
+      <c r="E462" s="1" t="inlineStr">
+        <is>
+          <t>買進(張)</t>
+        </is>
+      </c>
+      <c r="F462" s="1" t="inlineStr">
+        <is>
+          <t>賣出(張)</t>
+        </is>
+      </c>
+      <c r="G462" s="1" t="inlineStr">
+        <is>
+          <t>買進(萬元)</t>
+        </is>
+      </c>
+      <c r="H462" s="1" t="inlineStr">
+        <is>
+          <t>賣出(萬元)</t>
+        </is>
+      </c>
+      <c r="I462" s="1" t="inlineStr">
+        <is>
+          <t>淨買差(萬元)</t>
+        </is>
+      </c>
+      <c r="J462" s="1" t="inlineStr">
+        <is>
+          <t>買均</t>
+        </is>
+      </c>
+      <c r="K462" s="1" t="inlineStr">
+        <is>
+          <t>賣均</t>
+        </is>
+      </c>
+      <c r="L462" s="1" t="inlineStr">
+        <is>
+          <t>損益(萬)</t>
+        </is>
+      </c>
+    </row>
+    <row r="463" ht="16.5" customHeight="1">
+      <c r="B463" s="1" t="inlineStr">
+        <is>
+          <t>富邦-新竹</t>
+        </is>
+      </c>
+      <c r="C463" s="1" t="inlineStr">
+        <is>
+          <t>9647</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>台積電(2330)</t>
+        </is>
+      </c>
+      <c r="E463" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F463" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G463" s="3" t="n">
+        <v>7959</v>
+      </c>
+      <c r="H463" s="3" t="n">
+        <v>6776</v>
+      </c>
+      <c r="I463" s="3" t="n">
+        <v>1183</v>
+      </c>
+      <c r="J463" s="4" t="n">
+        <v>2273.89</v>
+      </c>
+      <c r="K463" s="4" t="n">
+        <v>2258.57</v>
+      </c>
+      <c r="L463" s="6">
+        <f>F463*(K463-J463)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="464" ht="16.5" customHeight="1">
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>群聯(8299)</t>
+        </is>
+      </c>
+      <c r="E464" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F464" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G464" s="3" t="n">
+        <v>7921</v>
+      </c>
+      <c r="H464" s="3" t="n">
+        <v>2336</v>
+      </c>
+      <c r="I464" s="3" t="n">
+        <v>5585</v>
+      </c>
+      <c r="J464" s="4" t="n">
+        <v>2400.18</v>
+      </c>
+      <c r="K464" s="4" t="n">
+        <v>2336.3</v>
+      </c>
+      <c r="L464" s="6">
+        <f>F464*(K464-J464)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="465" ht="16.5" customHeight="1">
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>華通(2313)</t>
+        </is>
+      </c>
+      <c r="E465" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="F465" s="3" t="n">
+        <v>166</v>
+      </c>
+      <c r="G465" s="3" t="n">
+        <v>5352</v>
+      </c>
+      <c r="H465" s="3" t="n">
+        <v>4610</v>
+      </c>
+      <c r="I465" s="3" t="n">
+        <v>742</v>
+      </c>
+      <c r="J465" s="4" t="n">
+        <v>277.3</v>
+      </c>
+      <c r="K465" s="4" t="n">
+        <v>277.73</v>
+      </c>
+      <c r="L465" s="5">
+        <f>F465*(K465-J465)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="466" ht="16.5" customHeight="1">
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>聯電(2303)</t>
+        </is>
+      </c>
+      <c r="E466" s="3" t="n">
+        <v>361</v>
+      </c>
+      <c r="F466" s="3" t="n">
+        <v>263</v>
+      </c>
+      <c r="G466" s="3" t="n">
+        <v>4151</v>
+      </c>
+      <c r="H466" s="3" t="n">
+        <v>3020</v>
+      </c>
+      <c r="I466" s="3" t="n">
+        <v>1131</v>
+      </c>
+      <c r="J466" s="4" t="n">
+        <v>114.99</v>
+      </c>
+      <c r="K466" s="4" t="n">
+        <v>114.81</v>
+      </c>
+      <c r="L466" s="6">
+        <f>F466*(K466-J466)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="467" ht="16.5" customHeight="1">
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>新代(7750)</t>
+        </is>
+      </c>
+      <c r="E467" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="F467" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G467" s="3" t="n">
+        <v>4138</v>
+      </c>
+      <c r="H467" s="3" t="n">
+        <v>590</v>
+      </c>
+      <c r="I467" s="3" t="n">
+        <v>3548</v>
+      </c>
+      <c r="J467" s="4" t="n">
+        <v>2433.88</v>
+      </c>
+      <c r="K467" s="4" t="n">
+        <v>2951.5</v>
+      </c>
+      <c r="L467" s="5">
+        <f>F467*(K467-J467)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="468" ht="16.5" customHeight="1">
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>主動統一台股增長(00981A)</t>
+        </is>
+      </c>
+      <c r="E468" s="3" t="n">
+        <v>1208</v>
+      </c>
+      <c r="F468" s="3" t="n">
+        <v>768</v>
+      </c>
+      <c r="G468" s="3" t="n">
+        <v>3601</v>
+      </c>
+      <c r="H468" s="3" t="n">
+        <v>2283</v>
+      </c>
+      <c r="I468" s="3" t="n">
+        <v>1318</v>
+      </c>
+      <c r="J468" s="4" t="n">
+        <v>29.81</v>
+      </c>
+      <c r="K468" s="4" t="n">
+        <v>29.73</v>
+      </c>
+      <c r="L468" s="6">
+        <f>F468*(K468-J468)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="469" ht="16.5" customHeight="1">
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>晶呈科技(4768)</t>
+        </is>
+      </c>
+      <c r="E469" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="F469" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G469" s="3" t="n">
+        <v>3053</v>
+      </c>
+      <c r="H469" s="3" t="n">
+        <v>1729</v>
+      </c>
+      <c r="I469" s="3" t="n">
+        <v>1324</v>
+      </c>
+      <c r="J469" s="4" t="n">
+        <v>455.66</v>
+      </c>
+      <c r="K469" s="4" t="n">
+        <v>455</v>
+      </c>
+      <c r="L469" s="6">
+        <f>F469*(K469-J469)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="470" ht="16.5" customHeight="1">
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>睿生光電(6861)</t>
+        </is>
+      </c>
+      <c r="E470" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="F470" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G470" s="3" t="n">
+        <v>2961</v>
+      </c>
+      <c r="H470" s="3" t="n">
+        <v>2086</v>
+      </c>
+      <c r="I470" s="3" t="n">
+        <v>875</v>
+      </c>
+      <c r="J470" s="4" t="n">
+        <v>448.58</v>
+      </c>
+      <c r="K470" s="4" t="n">
+        <v>453.54</v>
+      </c>
+      <c r="L470" s="5">
+        <f>F470*(K470-J470)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="471" ht="16.5" customHeight="1">
+      <c r="D471" s="2" t="inlineStr">
+        <is>
           <t>宜鼎(5289)</t>
         </is>
       </c>
-      <c r="E461" s="3" t="n">
+      <c r="E471" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="F461" s="3" t="n">
+      <c r="F471" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="G461" s="3" t="n">
+      <c r="G471" s="3" t="n">
         <v>2814</v>
       </c>
-      <c r="H461" s="3" t="n">
+      <c r="H471" s="3" t="n">
         <v>1264</v>
       </c>
-      <c r="I461" s="3" t="n">
+      <c r="I471" s="3" t="n">
         <v>1550</v>
       </c>
-      <c r="J461" s="4" t="n">
+      <c r="J471" s="4" t="n">
         <v>1758.44</v>
       </c>
-      <c r="K461" s="4" t="n">
+      <c r="K471" s="4" t="n">
         <v>1806</v>
       </c>
-      <c r="L461" s="5">
-        <f>F461*(K461-J461)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="462" ht="16.5" customHeight="1">
-      <c r="D462" s="2" t="inlineStr">
+      <c r="L471" s="5">
+        <f>F471*(K471-J471)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="472" ht="16.5" customHeight="1">
+      <c r="D472" s="2" t="inlineStr">
         <is>
           <t>頎邦(6147)</t>
         </is>
       </c>
-      <c r="E462" s="3" t="n">
+      <c r="E472" s="3" t="n">
         <v>126</v>
       </c>
-      <c r="F462" s="3" t="n">
+      <c r="F472" s="3" t="n">
         <v>84</v>
       </c>
-      <c r="G462" s="3" t="n">
+      <c r="G472" s="3" t="n">
         <v>2758</v>
       </c>
-      <c r="H462" s="3" t="n">
+      <c r="H472" s="3" t="n">
         <v>1834</v>
       </c>
-      <c r="I462" s="3" t="n">
+      <c r="I472" s="3" t="n">
         <v>924</v>
       </c>
-      <c r="J462" s="4" t="n">
+      <c r="J472" s="4" t="n">
         <v>218.87</v>
       </c>
-      <c r="K462" s="4" t="n">
+      <c r="K472" s="4" t="n">
         <v>218.3</v>
       </c>
-      <c r="L462" s="6">
-        <f>F462*(K462-J462)</f>
+      <c r="L472" s="6">
+        <f>F472*(K472-J472)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="97">
-    <mergeCell ref="B453:B462"/>
+    <mergeCell ref="B431:B450"/>
     <mergeCell ref="C189:C198"/>
     <mergeCell ref="B79:B88"/>
     <mergeCell ref="C387:C396"/>
+    <mergeCell ref="A452:A472"/>
     <mergeCell ref="C68:C77"/>
     <mergeCell ref="C310:C319"/>
     <mergeCell ref="B200:B209"/>
     <mergeCell ref="B90:B99"/>
-    <mergeCell ref="A442:A462"/>
     <mergeCell ref="C343:C352"/>
     <mergeCell ref="B145:B154"/>
     <mergeCell ref="C321:C330"/>
+    <mergeCell ref="C452:C461"/>
     <mergeCell ref="C200:C209"/>
     <mergeCell ref="B2:B11"/>
     <mergeCell ref="A376:A407"/>
-    <mergeCell ref="B431:B440"/>
     <mergeCell ref="C255:C264"/>
     <mergeCell ref="C46:C55"/>
     <mergeCell ref="A365:A374"/>
@@ -16561,6 +16881,7 @@
     <mergeCell ref="A244:A275"/>
     <mergeCell ref="B68:B77"/>
     <mergeCell ref="C244:C253"/>
+    <mergeCell ref="B463:B472"/>
     <mergeCell ref="A200:A242"/>
     <mergeCell ref="B266:B275"/>
     <mergeCell ref="C57:C66"/>
@@ -16570,7 +16891,6 @@
     <mergeCell ref="B321:B330"/>
     <mergeCell ref="C101:C110"/>
     <mergeCell ref="B233:B242"/>
-    <mergeCell ref="B442:B451"/>
     <mergeCell ref="B420:B429"/>
     <mergeCell ref="B134:B143"/>
     <mergeCell ref="B244:B253"/>
@@ -16591,17 +16911,17 @@
     <mergeCell ref="B189:B198"/>
     <mergeCell ref="C288:C297"/>
     <mergeCell ref="A288:A363"/>
-    <mergeCell ref="C431:C440"/>
     <mergeCell ref="C145:C154"/>
     <mergeCell ref="C24:C33"/>
     <mergeCell ref="C266:C275"/>
-    <mergeCell ref="A431:A440"/>
     <mergeCell ref="C156:C165"/>
     <mergeCell ref="B46:B55"/>
     <mergeCell ref="C79:C88"/>
     <mergeCell ref="B409:B418"/>
     <mergeCell ref="C90:C99"/>
+    <mergeCell ref="C463:C472"/>
     <mergeCell ref="B299:B308"/>
+    <mergeCell ref="B452:B461"/>
     <mergeCell ref="B376:B385"/>
     <mergeCell ref="C2:C11"/>
     <mergeCell ref="B310:B319"/>
@@ -16610,7 +16930,6 @@
     <mergeCell ref="B24:B33"/>
     <mergeCell ref="B365:B374"/>
     <mergeCell ref="C13:C22"/>
-    <mergeCell ref="C442:C451"/>
     <mergeCell ref="B222:B231"/>
     <mergeCell ref="B35:B44"/>
     <mergeCell ref="B277:B286"/>
@@ -16623,8 +16942,9 @@
     <mergeCell ref="C398:C407"/>
     <mergeCell ref="B13:B22"/>
     <mergeCell ref="C134:C143"/>
+    <mergeCell ref="A431:A450"/>
     <mergeCell ref="C211:C220"/>
-    <mergeCell ref="C453:C462"/>
+    <mergeCell ref="C431:C450"/>
     <mergeCell ref="C277:C286"/>
     <mergeCell ref="A145:A198"/>
     <mergeCell ref="C332:C341"/>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-05-23 15:27
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-05-22.xlsx
+++ b/data/reports/chip_radar_2026-05-22.xlsx
@@ -2530,29 +2530,29 @@
     <row r="58" ht="16.5" customHeight="1">
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>元大S＆P500(00646)</t>
+          <t>世界(5347)</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>4500</v>
+        <v>1203</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>33378</v>
+        <v>19400</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>0</v>
+        <v>195</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>33378</v>
+        <v>19205</v>
       </c>
       <c r="J58" s="4" t="n">
-        <v>74.17</v>
+        <v>161.27</v>
       </c>
       <c r="K58" s="4" t="n">
-        <v>0</v>
+        <v>162.25</v>
       </c>
       <c r="L58" s="5">
         <f>F58*(K58-J58)</f>
@@ -2562,29 +2562,29 @@
     <row r="59" ht="16.5" customHeight="1">
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>世界(5347)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>1203</v>
+        <v>236</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>19400</v>
+        <v>11989</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>195</v>
+        <v>1328</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>19205</v>
+        <v>10661</v>
       </c>
       <c r="J59" s="4" t="n">
-        <v>161.27</v>
+        <v>508.01</v>
       </c>
       <c r="K59" s="4" t="n">
-        <v>162.25</v>
+        <v>510.85</v>
       </c>
       <c r="L59" s="5">
         <f>F59*(K59-J59)</f>
@@ -2594,31 +2594,31 @@
     <row r="60" ht="16.5" customHeight="1">
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>金像電(2368)</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>236</v>
+        <v>79</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>11989</v>
+        <v>10463</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>1328</v>
+        <v>3</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>10661</v>
+        <v>10460</v>
       </c>
       <c r="J60" s="4" t="n">
-        <v>508.01</v>
+        <v>1324.39</v>
       </c>
       <c r="K60" s="4" t="n">
-        <v>510.85</v>
-      </c>
-      <c r="L60" s="5">
+        <v>27</v>
+      </c>
+      <c r="L60" s="6">
         <f>F60*(K60-J60)</f>
         <v/>
       </c>
@@ -2626,29 +2626,29 @@
     <row r="61" ht="16.5" customHeight="1">
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>金像電(2368)</t>
+          <t>南電(8046)</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>10463</v>
+        <v>8623</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>3</v>
+        <v>736</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>10460</v>
+        <v>7887</v>
       </c>
       <c r="J61" s="4" t="n">
-        <v>1324.39</v>
+        <v>947.59</v>
       </c>
       <c r="K61" s="4" t="n">
-        <v>27</v>
+        <v>919.62</v>
       </c>
       <c r="L61" s="6">
         <f>F61*(K61-J61)</f>
@@ -2658,31 +2658,31 @@
     <row r="62" ht="16.5" customHeight="1">
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>南電(8046)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>91</v>
+        <v>277</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>8623</v>
+        <v>8378</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>736</v>
+        <v>2395</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>7887</v>
+        <v>5983</v>
       </c>
       <c r="J62" s="4" t="n">
-        <v>947.59</v>
+        <v>302.46</v>
       </c>
       <c r="K62" s="4" t="n">
-        <v>919.62</v>
-      </c>
-      <c r="L62" s="6">
+        <v>315.08</v>
+      </c>
+      <c r="L62" s="5">
         <f>F62*(K62-J62)</f>
         <v/>
       </c>
@@ -2690,29 +2690,29 @@
     <row r="63" ht="16.5" customHeight="1">
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>聯陽(3014)</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>277</v>
+        <v>387</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>8378</v>
+        <v>5666</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>2395</v>
+        <v>0</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>5983</v>
+        <v>5666</v>
       </c>
       <c r="J63" s="4" t="n">
-        <v>302.46</v>
+        <v>146.41</v>
       </c>
       <c r="K63" s="4" t="n">
-        <v>315.08</v>
+        <v>0</v>
       </c>
       <c r="L63" s="5">
         <f>F63*(K63-J63)</f>
@@ -2722,31 +2722,31 @@
     <row r="64" ht="16.5" customHeight="1">
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>聯陽(3014)</t>
+          <t>台達電(2308)</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>387</v>
+        <v>18</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>5666</v>
+        <v>3821</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>5666</v>
+        <v>3715</v>
       </c>
       <c r="J64" s="4" t="n">
-        <v>146.41</v>
+        <v>2123</v>
       </c>
       <c r="K64" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L64" s="5">
+        <v>1065</v>
+      </c>
+      <c r="L64" s="6">
         <f>F64*(K64-J64)</f>
         <v/>
       </c>
@@ -2754,31 +2754,31 @@
     <row r="65" ht="16.5" customHeight="1">
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>台達電(2308)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>18</v>
+        <v>228</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>1</v>
+        <v>91</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>3821</v>
+        <v>2607</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>106</v>
+        <v>1043</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>3715</v>
+        <v>1564</v>
       </c>
       <c r="J65" s="4" t="n">
-        <v>2123</v>
+        <v>114.36</v>
       </c>
       <c r="K65" s="4" t="n">
-        <v>1065</v>
-      </c>
-      <c r="L65" s="6">
+        <v>114.6</v>
+      </c>
+      <c r="L65" s="5">
         <f>F65*(K65-J65)</f>
         <v/>
       </c>
@@ -2786,31 +2786,31 @@
     <row r="66" ht="16.5" customHeight="1">
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>聯電(2303)</t>
+          <t>威剛(3260)</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>228</v>
+        <v>49</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>91</v>
+        <v>36</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>2607</v>
+        <v>2066</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>1043</v>
+        <v>1491</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>1564</v>
+        <v>575</v>
       </c>
       <c r="J66" s="4" t="n">
-        <v>114.36</v>
+        <v>421.61</v>
       </c>
       <c r="K66" s="4" t="n">
-        <v>114.6</v>
-      </c>
-      <c r="L66" s="5">
+        <v>414.06</v>
+      </c>
+      <c r="L66" s="6">
         <f>F66*(K66-J66)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-05-23 16:44
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-05-22.xlsx
+++ b/data/reports/chip_radar_2026-05-22.xlsx
@@ -3925,29 +3925,29 @@
     <row r="98" ht="16.5" customHeight="1">
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>期街口布蘭特正2(00715L)</t>
+          <t>鑫科(3663)</t>
         </is>
       </c>
       <c r="E98" s="3" t="n">
-        <v>203</v>
+        <v>142</v>
       </c>
       <c r="F98" s="3" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>1265</v>
+        <v>1234</v>
       </c>
       <c r="H98" s="3" t="n">
-        <v>0</v>
+        <v>982</v>
       </c>
       <c r="I98" s="3" t="n">
-        <v>1265</v>
+        <v>252</v>
       </c>
       <c r="J98" s="4" t="n">
-        <v>62.3</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="K98" s="4" t="n">
-        <v>0</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="L98" s="5">
         <f>F98*(K98-J98)</f>
@@ -3957,29 +3957,29 @@
     <row r="99" ht="16.5" customHeight="1">
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>鑫科(3663)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E99" s="3" t="n">
-        <v>142</v>
+        <v>69</v>
       </c>
       <c r="F99" s="3" t="n">
-        <v>113</v>
+        <v>34</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>1234</v>
+        <v>1039</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>982</v>
+        <v>518</v>
       </c>
       <c r="I99" s="3" t="n">
-        <v>252</v>
+        <v>521</v>
       </c>
       <c r="J99" s="4" t="n">
-        <v>86.90000000000001</v>
+        <v>150.62</v>
       </c>
       <c r="K99" s="4" t="n">
-        <v>86.90000000000001</v>
+        <v>152.26</v>
       </c>
       <c r="L99" s="5">
         <f>F99*(K99-J99)</f>
@@ -4571,29 +4571,29 @@
     <row r="116" ht="16.5" customHeight="1">
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>元大台灣50正2(00631L)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E116" s="3" t="n">
-        <v>553</v>
+        <v>7</v>
       </c>
       <c r="F116" s="3" t="n">
-        <v>237</v>
+        <v>4</v>
       </c>
       <c r="G116" s="3" t="n">
-        <v>1763</v>
+        <v>1516</v>
       </c>
       <c r="H116" s="3" t="n">
-        <v>761</v>
+        <v>1008</v>
       </c>
       <c r="I116" s="3" t="n">
-        <v>1002</v>
+        <v>508</v>
       </c>
       <c r="J116" s="4" t="n">
-        <v>31.88</v>
+        <v>2165.29</v>
       </c>
       <c r="K116" s="4" t="n">
-        <v>32.12</v>
+        <v>2520.75</v>
       </c>
       <c r="L116" s="5">
         <f>F116*(K116-J116)</f>
@@ -4603,31 +4603,31 @@
     <row r="117" ht="16.5" customHeight="1">
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>國巨*(2327)</t>
         </is>
       </c>
       <c r="E117" s="3" t="n">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="F117" s="3" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G117" s="3" t="n">
-        <v>1516</v>
+        <v>1375</v>
       </c>
       <c r="H117" s="3" t="n">
-        <v>1008</v>
+        <v>667</v>
       </c>
       <c r="I117" s="3" t="n">
-        <v>508</v>
+        <v>708</v>
       </c>
       <c r="J117" s="4" t="n">
-        <v>2165.29</v>
+        <v>624.8200000000001</v>
       </c>
       <c r="K117" s="4" t="n">
-        <v>2520.75</v>
-      </c>
-      <c r="L117" s="5">
+        <v>606.36</v>
+      </c>
+      <c r="L117" s="6">
         <f>F117*(K117-J117)</f>
         <v/>
       </c>
@@ -4635,31 +4635,31 @@
     <row r="118" ht="16.5" customHeight="1">
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>國巨*(2327)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E118" s="3" t="n">
-        <v>22</v>
+        <v>301</v>
       </c>
       <c r="F118" s="3" t="n">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="G118" s="3" t="n">
-        <v>1375</v>
+        <v>1296</v>
       </c>
       <c r="H118" s="3" t="n">
-        <v>667</v>
+        <v>187</v>
       </c>
       <c r="I118" s="3" t="n">
-        <v>708</v>
+        <v>1109</v>
       </c>
       <c r="J118" s="4" t="n">
-        <v>624.8200000000001</v>
+        <v>43.06</v>
       </c>
       <c r="K118" s="4" t="n">
-        <v>606.36</v>
-      </c>
-      <c r="L118" s="6">
+        <v>44.52</v>
+      </c>
+      <c r="L118" s="5">
         <f>F118*(K118-J118)</f>
         <v/>
       </c>
@@ -4667,31 +4667,31 @@
     <row r="119" ht="16.5" customHeight="1">
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>雍智科技(6683)</t>
         </is>
       </c>
       <c r="E119" s="3" t="n">
-        <v>301</v>
+        <v>7</v>
       </c>
       <c r="F119" s="3" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="G119" s="3" t="n">
-        <v>1296</v>
+        <v>1212</v>
       </c>
       <c r="H119" s="3" t="n">
-        <v>187</v>
+        <v>166</v>
       </c>
       <c r="I119" s="3" t="n">
-        <v>1109</v>
+        <v>1046</v>
       </c>
       <c r="J119" s="4" t="n">
-        <v>43.06</v>
+        <v>1731.43</v>
       </c>
       <c r="K119" s="4" t="n">
-        <v>44.52</v>
-      </c>
-      <c r="L119" s="5">
+        <v>1655</v>
+      </c>
+      <c r="L119" s="6">
         <f>F119*(K119-J119)</f>
         <v/>
       </c>
@@ -4699,29 +4699,29 @@
     <row r="120" ht="16.5" customHeight="1">
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>雍智科技(6683)</t>
+          <t>今國光(6209)</t>
         </is>
       </c>
       <c r="E120" s="3" t="n">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="F120" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G120" s="3" t="n">
-        <v>1212</v>
+        <v>1064</v>
       </c>
       <c r="H120" s="3" t="n">
-        <v>166</v>
+        <v>41</v>
       </c>
       <c r="I120" s="3" t="n">
-        <v>1046</v>
+        <v>1023</v>
       </c>
       <c r="J120" s="4" t="n">
-        <v>1731.43</v>
+        <v>86.54000000000001</v>
       </c>
       <c r="K120" s="4" t="n">
-        <v>1655</v>
+        <v>81.2</v>
       </c>
       <c r="L120" s="6">
         <f>F120*(K120-J120)</f>
@@ -4731,29 +4731,29 @@
     <row r="121" ht="16.5" customHeight="1">
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>今國光(6209)</t>
+          <t>正新(2105)</t>
         </is>
       </c>
       <c r="E121" s="3" t="n">
-        <v>123</v>
+        <v>330</v>
       </c>
       <c r="F121" s="3" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="G121" s="3" t="n">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="H121" s="3" t="n">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="I121" s="3" t="n">
-        <v>1023</v>
+        <v>961</v>
       </c>
       <c r="J121" s="4" t="n">
-        <v>86.54000000000001</v>
+        <v>32.21</v>
       </c>
       <c r="K121" s="4" t="n">
-        <v>81.2</v>
+        <v>31.94</v>
       </c>
       <c r="L121" s="6">
         <f>F121*(K121-J121)</f>
@@ -5441,31 +5441,31 @@
     <row r="141" ht="16.5" customHeight="1">
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>凱基台灣TOP50(009816)</t>
+          <t>創意(3443)</t>
         </is>
       </c>
       <c r="E141" s="3" t="n">
-        <v>19939</v>
+        <v>54</v>
       </c>
       <c r="F141" s="3" t="n">
-        <v>140</v>
+        <v>11</v>
       </c>
       <c r="G141" s="3" t="n">
-        <v>28058</v>
+        <v>27526</v>
       </c>
       <c r="H141" s="3" t="n">
-        <v>198</v>
+        <v>5537</v>
       </c>
       <c r="I141" s="3" t="n">
-        <v>27860</v>
+        <v>21989</v>
       </c>
       <c r="J141" s="4" t="n">
-        <v>14.07</v>
+        <v>5097.39</v>
       </c>
       <c r="K141" s="4" t="n">
-        <v>14.14</v>
-      </c>
-      <c r="L141" s="5">
+        <v>5033.27</v>
+      </c>
+      <c r="L141" s="6">
         <f>F141*(K141-J141)</f>
         <v/>
       </c>
@@ -5473,29 +5473,29 @@
     <row r="142" ht="16.5" customHeight="1">
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>創意(3443)</t>
+          <t>臻鼎-KY(4958)</t>
         </is>
       </c>
       <c r="E142" s="3" t="n">
-        <v>54</v>
+        <v>506</v>
       </c>
       <c r="F142" s="3" t="n">
-        <v>11</v>
+        <v>267</v>
       </c>
       <c r="G142" s="3" t="n">
-        <v>27526</v>
+        <v>26089</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>5537</v>
+        <v>13765</v>
       </c>
       <c r="I142" s="3" t="n">
-        <v>21989</v>
+        <v>12324</v>
       </c>
       <c r="J142" s="4" t="n">
-        <v>5097.39</v>
+        <v>515.59</v>
       </c>
       <c r="K142" s="4" t="n">
-        <v>5033.27</v>
+        <v>515.53</v>
       </c>
       <c r="L142" s="6">
         <f>F142*(K142-J142)</f>
@@ -5505,29 +5505,29 @@
     <row r="143" ht="16.5" customHeight="1">
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>臻鼎-KY(4958)</t>
+          <t>南電(8046)</t>
         </is>
       </c>
       <c r="E143" s="3" t="n">
-        <v>506</v>
+        <v>274</v>
       </c>
       <c r="F143" s="3" t="n">
-        <v>267</v>
+        <v>78</v>
       </c>
       <c r="G143" s="3" t="n">
-        <v>26089</v>
+        <v>25615</v>
       </c>
       <c r="H143" s="3" t="n">
-        <v>13765</v>
+        <v>7278</v>
       </c>
       <c r="I143" s="3" t="n">
-        <v>12324</v>
+        <v>18337</v>
       </c>
       <c r="J143" s="4" t="n">
-        <v>515.59</v>
+        <v>934.84</v>
       </c>
       <c r="K143" s="4" t="n">
-        <v>515.53</v>
+        <v>933.09</v>
       </c>
       <c r="L143" s="6">
         <f>F143*(K143-J143)</f>
@@ -11227,29 +11227,29 @@
     <row r="307" ht="16.5" customHeight="1">
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>期街口布蘭特正2(00715L)</t>
+          <t>鑫科(3663)</t>
         </is>
       </c>
       <c r="E307" s="3" t="n">
-        <v>203</v>
+        <v>142</v>
       </c>
       <c r="F307" s="3" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="G307" s="3" t="n">
-        <v>1265</v>
+        <v>1234</v>
       </c>
       <c r="H307" s="3" t="n">
-        <v>0</v>
+        <v>982</v>
       </c>
       <c r="I307" s="3" t="n">
-        <v>1265</v>
+        <v>252</v>
       </c>
       <c r="J307" s="4" t="n">
-        <v>62.3</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="K307" s="4" t="n">
-        <v>0</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="L307" s="5">
         <f>F307*(K307-J307)</f>
@@ -11259,29 +11259,29 @@
     <row r="308" ht="16.5" customHeight="1">
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>鑫科(3663)</t>
+          <t>旺宏(2337)</t>
         </is>
       </c>
       <c r="E308" s="3" t="n">
-        <v>142</v>
+        <v>69</v>
       </c>
       <c r="F308" s="3" t="n">
-        <v>113</v>
+        <v>34</v>
       </c>
       <c r="G308" s="3" t="n">
-        <v>1234</v>
+        <v>1039</v>
       </c>
       <c r="H308" s="3" t="n">
-        <v>982</v>
+        <v>518</v>
       </c>
       <c r="I308" s="3" t="n">
-        <v>252</v>
+        <v>521</v>
       </c>
       <c r="J308" s="4" t="n">
-        <v>86.90000000000001</v>
+        <v>150.62</v>
       </c>
       <c r="K308" s="4" t="n">
-        <v>86.90000000000001</v>
+        <v>152.26</v>
       </c>
       <c r="L308" s="5">
         <f>F308*(K308-J308)</f>
@@ -15912,31 +15912,31 @@
     <row r="446" ht="16.5" customHeight="1">
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>期元大道瓊白銀(00738U)</t>
+          <t>智原(3035)</t>
         </is>
       </c>
       <c r="E446" s="3" t="n">
-        <v>240</v>
+        <v>68</v>
       </c>
       <c r="F446" s="3" t="n">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="G446" s="3" t="n">
-        <v>1476</v>
+        <v>1432</v>
       </c>
       <c r="H446" s="3" t="n">
-        <v>31</v>
+        <v>881</v>
       </c>
       <c r="I446" s="3" t="n">
-        <v>1445</v>
+        <v>551</v>
       </c>
       <c r="J446" s="4" t="n">
-        <v>61.49</v>
+        <v>210.59</v>
       </c>
       <c r="K446" s="4" t="n">
-        <v>62.4</v>
-      </c>
-      <c r="L446" s="5">
+        <v>209.79</v>
+      </c>
+      <c r="L446" s="6">
         <f>F446*(K446-J446)</f>
         <v/>
       </c>
@@ -15944,31 +15944,31 @@
     <row r="447" ht="16.5" customHeight="1">
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>智原(3035)</t>
+          <t>晶技(3042)</t>
         </is>
       </c>
       <c r="E447" s="3" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="F447" s="3" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G447" s="3" t="n">
-        <v>1432</v>
+        <v>1415</v>
       </c>
       <c r="H447" s="3" t="n">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="I447" s="3" t="n">
-        <v>551</v>
+        <v>530</v>
       </c>
       <c r="J447" s="4" t="n">
-        <v>210.59</v>
+        <v>176.91</v>
       </c>
       <c r="K447" s="4" t="n">
-        <v>209.79</v>
-      </c>
-      <c r="L447" s="6">
+        <v>176.92</v>
+      </c>
+      <c r="L447" s="5">
         <f>F447*(K447-J447)</f>
         <v/>
       </c>
@@ -15976,29 +15976,29 @@
     <row r="448" ht="16.5" customHeight="1">
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>晶技(3042)</t>
+          <t>敬鵬(2355)</t>
         </is>
       </c>
       <c r="E448" s="3" t="n">
-        <v>80</v>
+        <v>204</v>
       </c>
       <c r="F448" s="3" t="n">
-        <v>50</v>
+        <v>133</v>
       </c>
       <c r="G448" s="3" t="n">
-        <v>1415</v>
+        <v>1330</v>
       </c>
       <c r="H448" s="3" t="n">
-        <v>885</v>
+        <v>867</v>
       </c>
       <c r="I448" s="3" t="n">
-        <v>530</v>
+        <v>463</v>
       </c>
       <c r="J448" s="4" t="n">
-        <v>176.91</v>
+        <v>65.2</v>
       </c>
       <c r="K448" s="4" t="n">
-        <v>176.92</v>
+        <v>65.2</v>
       </c>
       <c r="L448" s="5">
         <f>F448*(K448-J448)</f>
@@ -16008,29 +16008,29 @@
     <row r="449" ht="16.5" customHeight="1">
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>敬鵬(2355)</t>
+          <t>中租-KY(5871)</t>
         </is>
       </c>
       <c r="E449" s="3" t="n">
-        <v>204</v>
+        <v>116</v>
       </c>
       <c r="F449" s="3" t="n">
-        <v>133</v>
+        <v>32</v>
       </c>
       <c r="G449" s="3" t="n">
-        <v>1330</v>
+        <v>1291</v>
       </c>
       <c r="H449" s="3" t="n">
-        <v>867</v>
+        <v>359</v>
       </c>
       <c r="I449" s="3" t="n">
-        <v>463</v>
+        <v>932</v>
       </c>
       <c r="J449" s="4" t="n">
-        <v>65.2</v>
+        <v>111.3</v>
       </c>
       <c r="K449" s="4" t="n">
-        <v>65.2</v>
+        <v>112.31</v>
       </c>
       <c r="L449" s="5">
         <f>F449*(K449-J449)</f>
@@ -16040,29 +16040,29 @@
     <row r="450" ht="16.5" customHeight="1">
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>中租-KY(5871)</t>
+          <t>上詮(3363)</t>
         </is>
       </c>
       <c r="E450" s="3" t="n">
-        <v>116</v>
+        <v>14</v>
       </c>
       <c r="F450" s="3" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="G450" s="3" t="n">
-        <v>1291</v>
+        <v>1162</v>
       </c>
       <c r="H450" s="3" t="n">
-        <v>359</v>
+        <v>550</v>
       </c>
       <c r="I450" s="3" t="n">
-        <v>932</v>
+        <v>612</v>
       </c>
       <c r="J450" s="4" t="n">
-        <v>111.3</v>
+        <v>830.29</v>
       </c>
       <c r="K450" s="4" t="n">
-        <v>112.31</v>
+        <v>916.33</v>
       </c>
       <c r="L450" s="5">
         <f>F450*(K450-J450)</f>
@@ -16696,29 +16696,29 @@
     <row r="468" ht="16.5" customHeight="1">
       <c r="D468" s="2" t="inlineStr">
         <is>
-          <t>主動統一台股增長(00981A)</t>
+          <t>晶呈科技(4768)</t>
         </is>
       </c>
       <c r="E468" s="3" t="n">
-        <v>1208</v>
+        <v>67</v>
       </c>
       <c r="F468" s="3" t="n">
-        <v>768</v>
+        <v>38</v>
       </c>
       <c r="G468" s="3" t="n">
-        <v>3601</v>
+        <v>3053</v>
       </c>
       <c r="H468" s="3" t="n">
-        <v>2283</v>
+        <v>1729</v>
       </c>
       <c r="I468" s="3" t="n">
-        <v>1318</v>
+        <v>1324</v>
       </c>
       <c r="J468" s="4" t="n">
-        <v>29.81</v>
+        <v>455.66</v>
       </c>
       <c r="K468" s="4" t="n">
-        <v>29.73</v>
+        <v>455</v>
       </c>
       <c r="L468" s="6">
         <f>F468*(K468-J468)</f>
@@ -16728,31 +16728,31 @@
     <row r="469" ht="16.5" customHeight="1">
       <c r="D469" s="2" t="inlineStr">
         <is>
-          <t>晶呈科技(4768)</t>
+          <t>睿生光電(6861)</t>
         </is>
       </c>
       <c r="E469" s="3" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F469" s="3" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G469" s="3" t="n">
-        <v>3053</v>
+        <v>2961</v>
       </c>
       <c r="H469" s="3" t="n">
-        <v>1729</v>
+        <v>2086</v>
       </c>
       <c r="I469" s="3" t="n">
-        <v>1324</v>
+        <v>875</v>
       </c>
       <c r="J469" s="4" t="n">
-        <v>455.66</v>
+        <v>448.58</v>
       </c>
       <c r="K469" s="4" t="n">
-        <v>455</v>
-      </c>
-      <c r="L469" s="6">
+        <v>453.54</v>
+      </c>
+      <c r="L469" s="5">
         <f>F469*(K469-J469)</f>
         <v/>
       </c>
@@ -16760,29 +16760,29 @@
     <row r="470" ht="16.5" customHeight="1">
       <c r="D470" s="2" t="inlineStr">
         <is>
-          <t>睿生光電(6861)</t>
+          <t>宜鼎(5289)</t>
         </is>
       </c>
       <c r="E470" s="3" t="n">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="F470" s="3" t="n">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="G470" s="3" t="n">
-        <v>2961</v>
+        <v>2814</v>
       </c>
       <c r="H470" s="3" t="n">
-        <v>2086</v>
+        <v>1264</v>
       </c>
       <c r="I470" s="3" t="n">
-        <v>875</v>
+        <v>1550</v>
       </c>
       <c r="J470" s="4" t="n">
-        <v>448.58</v>
+        <v>1758.44</v>
       </c>
       <c r="K470" s="4" t="n">
-        <v>453.54</v>
+        <v>1806</v>
       </c>
       <c r="L470" s="5">
         <f>F470*(K470-J470)</f>
@@ -16792,31 +16792,31 @@
     <row r="471" ht="16.5" customHeight="1">
       <c r="D471" s="2" t="inlineStr">
         <is>
-          <t>宜鼎(5289)</t>
+          <t>頎邦(6147)</t>
         </is>
       </c>
       <c r="E471" s="3" t="n">
-        <v>16</v>
+        <v>126</v>
       </c>
       <c r="F471" s="3" t="n">
-        <v>7</v>
+        <v>84</v>
       </c>
       <c r="G471" s="3" t="n">
-        <v>2814</v>
+        <v>2758</v>
       </c>
       <c r="H471" s="3" t="n">
-        <v>1264</v>
+        <v>1834</v>
       </c>
       <c r="I471" s="3" t="n">
-        <v>1550</v>
+        <v>924</v>
       </c>
       <c r="J471" s="4" t="n">
-        <v>1758.44</v>
+        <v>218.87</v>
       </c>
       <c r="K471" s="4" t="n">
-        <v>1806</v>
-      </c>
-      <c r="L471" s="5">
+        <v>218.3</v>
+      </c>
+      <c r="L471" s="6">
         <f>F471*(K471-J471)</f>
         <v/>
       </c>
@@ -16824,29 +16824,29 @@
     <row r="472" ht="16.5" customHeight="1">
       <c r="D472" s="2" t="inlineStr">
         <is>
-          <t>頎邦(6147)</t>
+          <t>矽格(6257)</t>
         </is>
       </c>
       <c r="E472" s="3" t="n">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="F472" s="3" t="n">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="G472" s="3" t="n">
-        <v>2758</v>
+        <v>2612</v>
       </c>
       <c r="H472" s="3" t="n">
-        <v>1834</v>
+        <v>1297</v>
       </c>
       <c r="I472" s="3" t="n">
-        <v>924</v>
+        <v>1315</v>
       </c>
       <c r="J472" s="4" t="n">
-        <v>218.87</v>
+        <v>227.17</v>
       </c>
       <c r="K472" s="4" t="n">
-        <v>218.3</v>
+        <v>223.67</v>
       </c>
       <c r="L472" s="6">
         <f>F472*(K472-J472)</f>

</xml_diff>